<commit_message>
Micro: fix 2024 cleaner false 'empty_workbook' skips — recover ~1,236 samples
Root cause of the 2024 -1,014 gap: the per-file emptiness probe opened workbooks
with openpyxl read_only=True, and ~20 Apr/Aug/etc. files omit the <dimension>
tag, so read_only reported ws.max_row = None → the check `not ws.max_row` treated
them as empty and silently skipped whole files (5,018 test rows / ~1,236 samples).
Fix: open the probe WITHOUT read_only (true dimension); genuinely-empty files
still skip via header-not-found.

Re-cleaned + enriched 2024: samples 8,094 -> 9,330 (official 9,108), tests
31,583 -> 36,461 (official 36,596, Δ -135), non-comp tests 3,407 -> 3,921
(official 3,928, Δ -7). Files skipped 20 -> 0. Rebuilt the combined dashboard
(20,894 rows) and regenerated the reconciliation / verification / classification
outputs. node --check clean.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/microbiology/reports/annual_reconciliation_to_fill.xlsx
+++ b/microbiology/reports/annual_reconciliation_to_fill.xlsx
@@ -728,28 +728,28 @@
         <v>641</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>448</v>
+        <v>520</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-193</v>
+        <v>-121</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>260</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>174</v>
+        <v>213</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>-86</v>
+        <v>-47</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>381</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>274</v>
+        <v>307</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>-107</v>
+        <v>-74</v>
       </c>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="5" t="n"/>
@@ -764,28 +764,28 @@
         <v>501</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>438</v>
+        <v>497</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>-63</v>
+        <v>-4</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>142</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-10</v>
+        <v>5</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>359</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>306</v>
+        <v>350</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>-53</v>
+        <v>-9</v>
       </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="5" t="n"/>
@@ -800,28 +800,28 @@
         <v>348</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>272</v>
+        <v>477</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>-76</v>
+        <v>129</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>128</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>113</v>
+        <v>196</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-15</v>
+        <v>68</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>220</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>159</v>
+        <v>281</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>-61</v>
+        <v>61</v>
       </c>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="n"/>
@@ -836,28 +836,28 @@
         <v>574</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>428</v>
+        <v>518</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>-146</v>
+        <v>-56</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>150</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>111</v>
+        <v>129</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-39</v>
+        <v>-21</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>424</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>317</v>
+        <v>389</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>-107</v>
+        <v>-35</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="5" t="n"/>
@@ -908,28 +908,28 @@
         <v>1483</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1342</v>
+        <v>1415</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>-141</v>
+        <v>-68</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>407</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>1076</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>903</v>
+        <v>960</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>-173</v>
+        <v>-116</v>
       </c>
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="5" t="n"/>
@@ -944,28 +944,28 @@
         <v>1425</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>773</v>
+        <v>1336</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>-652</v>
+        <v>-89</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>409</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>220</v>
+        <v>350</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-189</v>
+        <v>-59</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>1016</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>553</v>
+        <v>986</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>-463</v>
+        <v>-30</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="5" t="n"/>
@@ -980,28 +980,28 @@
         <v>504</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>434</v>
+        <v>608</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>-70</v>
+        <v>104</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>134</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>100</v>
+        <v>151</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-34</v>
+        <v>17</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>370</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>334</v>
+        <v>457</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>-36</v>
+        <v>87</v>
       </c>
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="5" t="n"/>
@@ -1124,28 +1124,28 @@
         <v>9108</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>8094</v>
+        <v>9330</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>-1014</v>
+        <v>222</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>2709</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>2464</v>
+        <v>2816</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>-245</v>
+        <v>107</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>6399</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>5630</v>
+        <v>6514</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>-769</v>
+        <v>115</v>
       </c>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="n"/>
@@ -1781,10 +1781,10 @@
         <v>9108</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>8094</v>
+        <v>9330</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-1014</v>
+        <v>222</v>
       </c>
       <c r="F2" s="5" t="n"/>
       <c r="G2" s="5" t="n"/>
@@ -1802,10 +1802,10 @@
         <v>6399</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>5547</v>
+        <v>6431</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>-852</v>
+        <v>32</v>
       </c>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
@@ -1823,10 +1823,10 @@
         <v>2709</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>2547</v>
+        <v>2899</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-162</v>
+        <v>190</v>
       </c>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
@@ -1844,10 +1844,10 @@
         <v>70.26000000000001</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>68.53</v>
+        <v>68.93000000000001</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-1.72</v>
+        <v>-1.33</v>
       </c>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>

</xml_diff>

<commit_message>
Micro: 2024 pipeline complete — dedup 13 barcodes + restore native GSO (enrich_gso)
Bake barcode de-dup into clean_2024 (13 cross-file re-exports removed: 9,330 ->
9,317). Re-ran the FULL pipeline incl. the enrich_gso step that was skipped last
time — restores gso_category_name_en etc., fixing the 2024 GSO regression
(Misc 564 -> 65, Fats -> 25, Jelly -> 120; native GSO on 7,846 rows). Dashboard
rebuilt (20,881 rows); workbooks + classification table regenerated. 2024 now
+209 vs official 9,108 (residual is date-basis, not duplicates).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/microbiology/reports/annual_reconciliation_to_fill.xlsx
+++ b/microbiology/reports/annual_reconciliation_to_fill.xlsx
@@ -692,10 +692,10 @@
         <v>653</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>220</v>
@@ -710,10 +710,10 @@
         <v>433</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K2" s="5" t="n"/>
       <c r="L2" s="5" t="n"/>
@@ -836,10 +836,10 @@
         <v>574</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>-56</v>
+        <v>-57</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>150</v>
@@ -854,10 +854,10 @@
         <v>424</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>-35</v>
+        <v>-36</v>
       </c>
       <c r="K6" s="5" t="n"/>
       <c r="L6" s="5" t="n"/>
@@ -944,28 +944,28 @@
         <v>1425</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1336</v>
+        <v>1333</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>-89</v>
+        <v>-92</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>409</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-59</v>
+        <v>-60</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>1016</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>-30</v>
+        <v>-32</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="5" t="n"/>
@@ -1088,28 +1088,28 @@
         <v>834</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>832</v>
+        <v>825</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>-2</v>
+        <v>-9</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>199</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H13" s="4" t="n">
         <v>635</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>626</v>
+        <v>620</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>-9</v>
+        <v>-15</v>
       </c>
       <c r="K13" s="5" t="n"/>
       <c r="L13" s="5" t="n"/>
@@ -1124,28 +1124,28 @@
         <v>9108</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>9330</v>
+        <v>9317</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>222</v>
+        <v>209</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>2709</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>2816</v>
+        <v>2814</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>6399</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>6514</v>
+        <v>6503</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="n"/>
@@ -1781,10 +1781,10 @@
         <v>9108</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>9330</v>
+        <v>9317</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>222</v>
+        <v>209</v>
       </c>
       <c r="F2" s="5" t="n"/>
       <c r="G2" s="5" t="n"/>
@@ -1802,10 +1802,10 @@
         <v>6399</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>6431</v>
+        <v>6420</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
@@ -1823,10 +1823,10 @@
         <v>2709</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>2899</v>
+        <v>2897</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
@@ -1844,10 +1844,10 @@
         <v>70.26000000000001</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>68.93000000000001</v>
+        <v>68.91</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-1.33</v>
+        <v>-1.35</v>
       </c>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>

</xml_diff>